<commit_message>
[Feat] 엘리트 번개 포탑 패시브 구현 (KnockbackOnHit, ScaleProjectile)
- KnockbackOnHitPassive.cs: 피격 시 넉백 패시브 신규 구현
- ScaleProjectilePassive.cs: 투사체 크기 배율 패시브 신규 구현
- Projectile.cs: SetRuntimeShove / SetModelScale 런타임 주입 메서드 추가
- TriggerHandle.cs: hasStunEffect / stunDuration 스턴 이펙트 지원 추가
- TurretTrain.cs: ProjectileModelScale / ProjectileKnockbackPower/Duration 프로퍼티 추가 및 발사 시 적용
- TrainPassiveSkillFactory.cs: KnockbackOnHitPassive, ScaleProjectilePassive 팩토리 등록
- DB.asset / TrainSkillData.xlsx: 엘리트 번개 투사체 ID, 60013 패시브 데이터 반영
</commit_message>
<xml_diff>
--- a/Assets/02_Resources/Data/TrainSkillData.xlsx
+++ b/Assets/02_Resources/Data/TrainSkillData.xlsx
@@ -892,15 +892,25 @@
           <t>5초 동안 강력한 포격을 퍼붓습니다.</t>
         </is>
       </c>
-      <c r="D6" s="21" t="n"/>
-      <c r="E6" s="21" t="n"/>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>SelfBuff</t>
+        </is>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>30</v>
+      </c>
       <c r="H6" s="21" t="n"/>
       <c r="I6" s="21" t="n"/>
       <c r="J6" s="21" t="n"/>
       <c r="K6" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="L6" s="21" t="n"/>
+      <c r="L6" s="21" t="inlineStr">
+        <is>
+          <t>AttackInterval:-80|AttackDamage:100</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="21" t="n"/>

</xml_diff>

<commit_message>
[Refactor] 과충전 AttackCount 통합 + 정수 스탯 flat 표기 전환
- TurretTrain.cs·RangeTrain.cs: StatModifier의 AttackCount/TargetCount를 base 비례 % → flat +N으로 변경, 미사용 accumulator 제거
- DB.asset: 과충전(60011) RepeatAfterAttack 제거 → StatModifier:AttackCount:2:AttackInterval:30 (공속 페널티 40→30%)
- DB.asset: 과부하(60013) TargetCount:100 → TargetCount:2 (실효 동일)
- TrainSkillData.xlsx: DB 동기화 (sheet2 C12·F14)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Assets/02_Resources/Data/TrainSkillData.xlsx
+++ b/Assets/02_Resources/Data/TrainSkillData.xlsx
@@ -265,7 +265,7 @@
     <t xml:space="preserve">StatModifier:AttackDamage:100|ScaleProjectile</t>
   </si>
   <si>
-    <t xml:space="preserve">RepeatAfterAttack:0.2:2|StatModifier:AttackInterval:40</t>
+    <t xml:space="preserve">StatModifier:AttackCount:2:AttackInterval:30</t>
   </si>
   <si>
     <t xml:space="preserve">Strengthen:100|StatModifier:AttackArea:50</t>
@@ -316,7 +316,7 @@
     <t xml:space="preserve">skill_projectile_prefab_id</t>
   </si>
   <si>
-    <t>TargetCount:100</t>
+    <t>TargetCount:2</t>
   </si>
   <si>
     <t>AttackArea:-30:AttackRange:50</t>

</xml_diff>